<commit_message>
feat: LO differential oracle (1634 cases, 89.1% agreement), residual functions, 95%+ test coverage
Oracle: benchmarks/oracle-cases.json + run_oracle.sh + agreement.json +
docs/AGREEMENT.md — per-function ironcalc-vs-LibreOffice value agreement
with Excel-as-arbiter triage; 5 strong ironcalc bug candidates and 4
LO-deviates-Excel cases documented. Residual engine functions in vendored
master: ENCODEURL (RFC 3986), HYPERLINK (value semantics), AGGREGATE
(function_nums 1-19, full options bitmask incl. hidden rows via SUBTOTAL's
visibility path). Coverage 497/522 (95.2%). All benchmarks regenerated for
the master engine (perf neutral; LO 15-vs-17-sig-digit cache drift and
openpyxl's 101,961 stripped caches now quantified). xlq code coverage:
every src file >=95% lines (cargo-llvm-cov, 21 tests added, 67 total).
17 review findings fixed. Full-catalog semantics spec added
(docs/specs/full-catalog-semantics.md).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/branch-consolidation.xlsx
+++ b/fixtures/branch-consolidation.xlsx
@@ -15,6 +15,28 @@
   <definedNames/>
   <calcPr/>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -116,9 +138,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="1">
     <font>
-      <sz val="13"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <sz val="12"/>
+      <name val="Inter"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -141,7 +162,7 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1" applyFill="1"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
     <xf xfId="0" borderId="0" fillId="0" fontId="0" numFmtId="0"/>
@@ -153,6 +174,321 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4472C4"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="020F0302020204030204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M16"/>

</xml_diff>